<commit_message>
Refresh event data (Sun 09/13/2026 09:51)
First full refresh since the scraper fixes landed. All 46 sources
succeeded - failures: none, and the failure log is now completely
empty for the first time. La Mesa Village failed its first attempt
and recovered on the retry.

1735 events (1723 upcoming), 294 newly added since the 09/04 build.
The venues fixed last session are all producing listings again:
McGuffie's 79, Humphrey's Concerts 13, Lou Lou's 4, Worldbeat 3.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/scraper/failure_log.xlsx
+++ b/scraper/failure_log.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,31 +441,6 @@
       <c r="E1" t="inlineStr">
         <is>
           <t>Last Failed</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Worldbeat Center</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>NoEventsFound</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>scraper returned 0 events</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>11</v>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>2026-09-04 07:46</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refresh event data (Fri 09/25/2026 15:03)
Automated data refresh via update-events.bat

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/scraper/failure_log.xlsx
+++ b/scraper/failure_log.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,6 +441,31 @@
       <c r="E1" t="inlineStr">
         <is>
           <t>Last Failed</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Brick By Brick</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>NoEventsFound</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>scraper returned 0 events</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>2026-09-25 15:01</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refresh event data (Mon 09/28/2026 14:43)
Automated data refresh via update-events.bat

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/scraper/failure_log.xlsx
+++ b/scraper/failure_log.xlsx
@@ -461,11 +461,11 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-09-25 15:01</t>
+          <t>2026-09-28 14:41</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refresh event data (Wed 10/14/2026 21:00)
Automated data refresh via update-events.bat

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/scraper/failure_log.xlsx
+++ b/scraper/failure_log.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -461,11 +461,136 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-09-28 14:41</t>
+          <t>2026-10-14 20:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Casbah</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>HTTP 403</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>403 Client Error: Forbidden for url: https://www.casbahmusic.com/</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2026-10-14 20:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Del Mar Fairgrounds</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>NoEventsFound</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>scraper returned 0 events</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2026-10-14 20:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Lou Lou's Jungle Room</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>HTTP 403</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>403 Client Error: Forbidden for url: https://www.casbahmusic.com/venues/lou-lous/</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>2026-10-14 20:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Museum of Making Music</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>NoEventsFound</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>scraper returned 0 events</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>2026-10-14 20:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Quartyard</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>HTTP 403</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>403 Client Error: Forbidden for url: https://www.casbahmusic.com/</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>2026-10-14 20:58</t>
         </is>
       </c>
     </row>
@@ -480,7 +605,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -510,6 +635,31 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Brick By Brick</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>NoEventsFound</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>scraper returned 0 events</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>2026-10-14 20:58</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>